<commit_message>
Figure tidy up mostly
</commit_message>
<xml_diff>
--- a/Data/species_TL.xlsx
+++ b/Data/species_TL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Multispecies_model\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4AD86F4-4599-435D-AEF9-8699831CC448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9643480A-1E5E-4505-8A36-9ED98C1B87AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-16110" windowWidth="29040" windowHeight="15720" xr2:uid="{2705465D-B030-4ADC-B1AE-6554A68AC405}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="63">
   <si>
     <t xml:space="preserve">Stock </t>
   </si>
@@ -101,81 +101,42 @@
     <t>ICES HAWG_NS 2r_Ammodytes_marinus</t>
   </si>
   <si>
-    <t>Sprattus sprattus</t>
-  </si>
-  <si>
     <t>S.sprattus</t>
   </si>
   <si>
-    <t>Clupea harengus</t>
-  </si>
-  <si>
     <t>C.harengus</t>
   </si>
   <si>
-    <t>Ammodytes marinus</t>
-  </si>
-  <si>
     <t>A. marinus</t>
   </si>
   <si>
-    <t>Trisopterus esmarki</t>
-  </si>
-  <si>
     <t>T. esmarki</t>
   </si>
   <si>
-    <t>Pleuronectes platessa</t>
-  </si>
-  <si>
     <t>P. platessa</t>
   </si>
   <si>
-    <t>Pollachius virens</t>
-  </si>
-  <si>
     <t>P. virens</t>
   </si>
   <si>
-    <t>Glyptocephalus cynoglossus</t>
-  </si>
-  <si>
     <t>G. cynoglossus</t>
   </si>
   <si>
-    <t>Solea solea</t>
-  </si>
-  <si>
     <t>S. solea</t>
   </si>
   <si>
-    <t>Gadus morhua</t>
-  </si>
-  <si>
     <t>G. morhua</t>
   </si>
   <si>
-    <t>Scopthalmus maximus</t>
-  </si>
-  <si>
-    <t>Melanogrammus aeglefinus</t>
-  </si>
-  <si>
     <t>M. aeglefinus</t>
   </si>
   <si>
-    <t>Merlangius merlangus</t>
-  </si>
-  <si>
     <t>M. merlangus</t>
   </si>
   <si>
     <t>common</t>
   </si>
   <si>
-    <t>Species</t>
-  </si>
-  <si>
     <t>S.short</t>
   </si>
   <si>
@@ -216,13 +177,61 @@
   </si>
   <si>
     <t>Haddock</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>1r</t>
+  </si>
+  <si>
+    <t>2r</t>
+  </si>
+  <si>
+    <t>3r</t>
+  </si>
+  <si>
+    <t>7d</t>
+  </si>
+  <si>
+    <t>NS</t>
+  </si>
+  <si>
+    <t>NW</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Viking</t>
+  </si>
+  <si>
+    <t>4-3a-7d</t>
+  </si>
+  <si>
+    <t>4-6-3a</t>
+  </si>
+  <si>
+    <t>4-20</t>
+  </si>
+  <si>
+    <t>troph.cat</t>
+  </si>
+  <si>
+    <t>4.1-4.9</t>
+  </si>
+  <si>
+    <t>≤ 4.0</t>
+  </si>
+  <si>
+    <t>≥ 5.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,6 +252,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -293,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -305,6 +320,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -639,13 +656,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8258E3A5-6D7B-4A73-A0F9-7FE12D8D1C0F}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="71" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -653,101 +670,119 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D1" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+      <c r="F1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B2">
-        <v>3.99</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B3">
-        <v>3.99</v>
-      </c>
-      <c r="C3" t="s">
-        <v>25</v>
+        <v>4</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="F3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>3.99</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
+        <v>4</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B5">
         <v>3.8</v>
       </c>
-      <c r="C5" t="s">
-        <v>23</v>
+      <c r="C5" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>3.99</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
+        <v>4</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -755,16 +790,19 @@
         <v>4.3</v>
       </c>
       <c r="C7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" t="s">
         <v>21</v>
       </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
       <c r="E7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -772,16 +810,19 @@
         <v>4.2</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -789,16 +830,19 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -806,33 +850,39 @@
         <v>4.5</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>3.99</v>
-      </c>
-      <c r="C11" t="s">
-        <v>33</v>
+        <v>4</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -840,33 +890,39 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B13">
         <v>5</v>
       </c>
-      <c r="C13" t="s">
-        <v>35</v>
+      <c r="C13" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -874,84 +930,99 @@
         <v>4.5</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+      <c r="F14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B15">
         <v>5</v>
       </c>
-      <c r="C15" t="s">
-        <v>35</v>
+      <c r="C15" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E15" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+      <c r="F15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B16">
         <v>5.2</v>
       </c>
-      <c r="C16" t="s">
-        <v>37</v>
+      <c r="C16" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B17">
         <v>5.2</v>
       </c>
-      <c r="C17" t="s">
-        <v>37</v>
+      <c r="C17" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+      <c r="F17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B18">
         <v>5.2</v>
       </c>
-      <c r="C18" t="s">
-        <v>37</v>
+      <c r="C18" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+      <c r="F18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -959,34 +1030,41 @@
         <v>4.7</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="F19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B20">
         <v>5.3</v>
       </c>
-      <c r="C20" t="s">
-        <v>42</v>
+      <c r="C20" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="E20" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" t="s">
         <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;R&amp;"Calibri"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
   </headerFooter>

</xml_diff>